<commit_message>
Restaurer la formule de loi de puissance sur OPEX Guarantees & prev maint
La COPEX Library/le BP reintroduisent la loi de puissance sur ce poste,
cette fois en texte descriptif ("794,13 x MWh^(-0,61) k€/MWh") plutot qu'en
formule Excel executable (plus de reference externe cassante a chaque
install). Nouveau parseur _TEXT_POWER_LAW_FORMULA, meme coefficient/exposant
et meme interpretation que l'ancienne formule (ordre de grandeur verifie).

Le prorata au-dela de 15 ans (20 ans -> x1,33, 30 ans -> x2) est deja le
comportement du moteur par construction (taux annualise applique chaque
annee de la vie du projet) - verrouille par un nouveau test, aucun
changement de code necessaire sur ce point.

415 tests passent.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bankability_app/config/copex_icp.xlsx
+++ b/bankability_app/config/copex_icp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julien.borgescosta\Videos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B087308-E673-4E16-9417-C0D7ADF59DAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53138118-6231-4F0B-A583-C1B70DE1B40E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{540C8C1F-1E50-4CA0-A325-996E2020A5FA}"/>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3794E96B-8F3C-4BC8-B883-5D97263E2710}"/>
@@ -163,7 +163,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="58">
   <si>
     <t>Hypothèses CAPEX BP - BESS Standalone</t>
   </si>
@@ -291,15 +291,9 @@
     <t>Insurances construction (% of Total Capex)</t>
   </si>
   <si>
-    <t>OPEX - Guarantees &amp; prev maint - 4h (annual)</t>
-  </si>
-  <si>
     <t>Insurances operation (% Capex + 1y incomes)</t>
   </si>
   <si>
-    <t>OPEX - Guarantees &amp; prev maint - 2h</t>
-  </si>
-  <si>
     <t>Asset Management construction (incl. Coût fixe ISA)</t>
   </si>
   <si>
@@ -331,6 +325,18 @@
   </si>
   <si>
     <t>V1 - JBO - 08/10/2026</t>
+  </si>
+  <si>
+    <t>794,13 × MWh^(-0,61) k€/MWh</t>
+  </si>
+  <si>
+    <t>1 408 × MWh^(-0,891) k€/MWh</t>
+  </si>
+  <si>
+    <t>OPEX - Guarantees &amp; prev maint - 2h (15y)</t>
+  </si>
+  <si>
+    <t>OPEX - Guarantees &amp; prev maint - 4h (15 y)</t>
   </si>
 </sst>
 </file>
@@ -345,12 +351,19 @@
     <numFmt numFmtId="167" formatCode="#,##0&quot; k€&quot;"/>
     <numFmt numFmtId="168" formatCode="#,##0&quot; k€/MWh/y&quot;"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1246,347 +1259,351 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="9">
+  <cellStyleXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="19" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="7"/>
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="7" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="7" borderId="2" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="7"/>
-    <xf numFmtId="167" fontId="5" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="6" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="16" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="30" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="31" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="32" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="6" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="36" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="7" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="37" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="7" borderId="2" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="7" borderId="2" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="38" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="7" borderId="38" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="7" borderId="32" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="7" borderId="32" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="7" borderId="32" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="7" borderId="33" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="7" borderId="34" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="4" fillId="6" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="6" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="39" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="6" borderId="35" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="6" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="6" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="42" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="45" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="46" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="47" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="7" borderId="47" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="7" borderId="35" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="7" borderId="35" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="7" borderId="35" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="7" borderId="40" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="42" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="44" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="45" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="10" borderId="48" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="10" borderId="49" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="10" borderId="50" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="15" fontId="18" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="18" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="18" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="15" fontId="17" fillId="5" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="17" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="17" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="5" fillId="6" borderId="30" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="6" borderId="31" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="6" borderId="32" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="6" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="36" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="7" borderId="47" xfId="9" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="37" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="7" borderId="1" xfId="9" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="38" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="7" borderId="38" xfId="9" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="7" borderId="38" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="7" borderId="32" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="7" borderId="32" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="7" borderId="32" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="7" borderId="33" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="7" borderId="34" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="3" fillId="6" borderId="33" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="3" fillId="6" borderId="34" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="6" borderId="39" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="6" borderId="35" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="6" borderId="35" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="6" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="41" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="42" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="45" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="46" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="47" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="7" borderId="47" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="7" borderId="35" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="7" borderId="35" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="7" borderId="35" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="7" borderId="40" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="42" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="43" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="44" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="44" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="44" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="45" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="10" borderId="48" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="10" borderId="49" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="10" borderId="50" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="9">
+  <cellStyles count="10">
     <cellStyle name="Lien hypertexte" xfId="7" builtinId="8"/>
     <cellStyle name="Milliers 2" xfId="6" xr:uid="{165C533B-3352-44B4-8816-FA61A1D4443F}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 7 2 2" xfId="2" xr:uid="{59B154AF-C098-49BC-876B-3A59780822FF}"/>
+    <cellStyle name="Normal 7 2 2 5" xfId="9" xr:uid="{EFDEDC34-84D1-4D69-A1B4-469F6B574776}"/>
     <cellStyle name="Normal 8" xfId="1" xr:uid="{7FC3F739-C4F8-4AA1-9803-29F0CCFF569C}"/>
     <cellStyle name="Normal 8 3" xfId="4" xr:uid="{7A6CD391-1E01-4093-B624-EC1750B53C5E}"/>
     <cellStyle name="Normal 8 4" xfId="8" xr:uid="{AC17045E-1BE2-4209-AA5C-A0A7201318D0}"/>
@@ -2158,8 +2175,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="12" customHeight="1" thickBot="1">
-      <c r="A1" s="49"/>
-      <c r="B1" s="49"/>
+      <c r="A1" s="98"/>
+      <c r="B1" s="98"/>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
       <c r="E1" s="14"/>
@@ -2168,43 +2185,43 @@
     </row>
     <row r="2" spans="1:8" ht="43.15" customHeight="1" thickBot="1">
       <c r="A2" s="14"/>
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="108" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="55"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="109"/>
+      <c r="E2" s="109"/>
+      <c r="F2" s="109"/>
+      <c r="G2" s="110"/>
     </row>
     <row r="3" spans="1:8" ht="17.25">
       <c r="A3" s="14"/>
-      <c r="B3" s="56" t="s">
+      <c r="B3" s="99" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="57"/>
-      <c r="E3" s="57"/>
-      <c r="F3" s="57"/>
-      <c r="G3" s="58"/>
+      <c r="C3" s="100"/>
+      <c r="D3" s="100"/>
+      <c r="E3" s="100"/>
+      <c r="F3" s="100"/>
+      <c r="G3" s="101"/>
     </row>
     <row r="4" spans="1:8" ht="17.25">
       <c r="A4" s="14"/>
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="102" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="60"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
-      <c r="F4" s="60"/>
-      <c r="G4" s="61"/>
+      <c r="C4" s="103"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="103"/>
+      <c r="F4" s="103"/>
+      <c r="G4" s="104"/>
       <c r="H4" s="28" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" thickBot="1">
-      <c r="A5" s="49"/>
-      <c r="B5" s="49"/>
+      <c r="A5" s="98"/>
+      <c r="B5" s="98"/>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
@@ -2213,14 +2230,14 @@
     </row>
     <row r="6" spans="1:8" ht="18" thickBot="1">
       <c r="A6" s="14"/>
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="105" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="51"/>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
-      <c r="G6" s="52"/>
+      <c r="C6" s="106"/>
+      <c r="D6" s="106"/>
+      <c r="E6" s="106"/>
+      <c r="F6" s="106"/>
+      <c r="G6" s="107"/>
     </row>
     <row r="7" spans="1:8" ht="17.25">
       <c r="A7" s="14"/>
@@ -2658,571 +2675,694 @@
       <c r="G47" s="19"/>
     </row>
     <row r="57" spans="1:2" ht="17.25">
-      <c r="A57" s="49"/>
-      <c r="B57" s="49"/>
+      <c r="A57" s="98"/>
+      <c r="B57" s="98"/>
     </row>
     <row r="58" spans="1:2" ht="17.25">
-      <c r="A58" s="49"/>
-      <c r="B58" s="49"/>
+      <c r="A58" s="98"/>
+      <c r="B58" s="98"/>
     </row>
     <row r="59" spans="1:2" ht="17.25">
-      <c r="A59" s="49"/>
-      <c r="B59" s="49"/>
+      <c r="A59" s="98"/>
+      <c r="B59" s="98"/>
     </row>
     <row r="60" spans="1:2" ht="17.25">
-      <c r="A60" s="49"/>
-      <c r="B60" s="49"/>
+      <c r="A60" s="98"/>
+      <c r="B60" s="98"/>
     </row>
     <row r="61" spans="1:2" ht="17.25">
-      <c r="A61" s="49"/>
-      <c r="B61" s="49"/>
+      <c r="A61" s="98"/>
+      <c r="B61" s="98"/>
     </row>
     <row r="62" spans="1:2" ht="17.25">
-      <c r="A62" s="49"/>
-      <c r="B62" s="49"/>
+      <c r="A62" s="98"/>
+      <c r="B62" s="98"/>
     </row>
     <row r="63" spans="1:2" ht="17.25">
-      <c r="A63" s="49"/>
-      <c r="B63" s="49"/>
+      <c r="A63" s="98"/>
+      <c r="B63" s="98"/>
     </row>
     <row r="64" spans="1:2" ht="17.25">
-      <c r="A64" s="49"/>
-      <c r="B64" s="49"/>
+      <c r="A64" s="98"/>
+      <c r="B64" s="98"/>
     </row>
     <row r="65" spans="1:2" ht="17.25">
-      <c r="A65" s="49"/>
-      <c r="B65" s="49"/>
+      <c r="A65" s="98"/>
+      <c r="B65" s="98"/>
     </row>
     <row r="66" spans="1:2" ht="17.25">
-      <c r="A66" s="49"/>
-      <c r="B66" s="49"/>
+      <c r="A66" s="98"/>
+      <c r="B66" s="98"/>
     </row>
     <row r="67" spans="1:2" ht="17.25">
-      <c r="A67" s="49"/>
-      <c r="B67" s="49"/>
+      <c r="A67" s="98"/>
+      <c r="B67" s="98"/>
     </row>
     <row r="68" spans="1:2" ht="17.25">
-      <c r="A68" s="49"/>
-      <c r="B68" s="49"/>
+      <c r="A68" s="98"/>
+      <c r="B68" s="98"/>
     </row>
     <row r="69" spans="1:2" ht="17.25">
-      <c r="A69" s="49"/>
-      <c r="B69" s="49"/>
+      <c r="A69" s="98"/>
+      <c r="B69" s="98"/>
     </row>
     <row r="70" spans="1:2" ht="17.25">
-      <c r="A70" s="49"/>
-      <c r="B70" s="49"/>
+      <c r="A70" s="98"/>
+      <c r="B70" s="98"/>
     </row>
     <row r="71" spans="1:2" ht="17.25">
-      <c r="A71" s="49"/>
-      <c r="B71" s="49"/>
+      <c r="A71" s="98"/>
+      <c r="B71" s="98"/>
     </row>
     <row r="72" spans="1:2" ht="17.25">
-      <c r="A72" s="49"/>
-      <c r="B72" s="49"/>
+      <c r="A72" s="98"/>
+      <c r="B72" s="98"/>
     </row>
     <row r="73" spans="1:2" ht="17.25">
-      <c r="A73" s="49"/>
-      <c r="B73" s="49"/>
+      <c r="A73" s="98"/>
+      <c r="B73" s="98"/>
     </row>
     <row r="74" spans="1:2" ht="17.25">
-      <c r="A74" s="49"/>
-      <c r="B74" s="49"/>
+      <c r="A74" s="98"/>
+      <c r="B74" s="98"/>
     </row>
     <row r="75" spans="1:2" ht="17.25">
-      <c r="A75" s="49"/>
-      <c r="B75" s="49"/>
+      <c r="A75" s="98"/>
+      <c r="B75" s="98"/>
     </row>
     <row r="76" spans="1:2" ht="17.25">
-      <c r="A76" s="49"/>
-      <c r="B76" s="49"/>
+      <c r="A76" s="98"/>
+      <c r="B76" s="98"/>
     </row>
     <row r="77" spans="1:2" ht="17.25">
-      <c r="A77" s="49"/>
-      <c r="B77" s="49"/>
+      <c r="A77" s="98"/>
+      <c r="B77" s="98"/>
     </row>
     <row r="78" spans="1:2" ht="17.25">
-      <c r="A78" s="49"/>
-      <c r="B78" s="49"/>
+      <c r="A78" s="98"/>
+      <c r="B78" s="98"/>
     </row>
     <row r="79" spans="1:2" ht="17.25">
-      <c r="A79" s="49"/>
-      <c r="B79" s="49"/>
+      <c r="A79" s="98"/>
+      <c r="B79" s="98"/>
     </row>
     <row r="80" spans="1:2" ht="17.25">
-      <c r="A80" s="49"/>
-      <c r="B80" s="49"/>
+      <c r="A80" s="98"/>
+      <c r="B80" s="98"/>
     </row>
     <row r="81" spans="1:2" ht="17.25">
-      <c r="A81" s="49"/>
-      <c r="B81" s="49"/>
+      <c r="A81" s="98"/>
+      <c r="B81" s="98"/>
     </row>
     <row r="82" spans="1:2" ht="17.25">
-      <c r="A82" s="49"/>
-      <c r="B82" s="49"/>
+      <c r="A82" s="98"/>
+      <c r="B82" s="98"/>
     </row>
     <row r="83" spans="1:2" ht="17.25">
-      <c r="A83" s="49"/>
-      <c r="B83" s="49"/>
+      <c r="A83" s="98"/>
+      <c r="B83" s="98"/>
     </row>
     <row r="84" spans="1:2" ht="17.25">
-      <c r="A84" s="49"/>
-      <c r="B84" s="49"/>
+      <c r="A84" s="98"/>
+      <c r="B84" s="98"/>
     </row>
     <row r="85" spans="1:2" ht="17.25">
-      <c r="A85" s="49"/>
-      <c r="B85" s="49"/>
+      <c r="A85" s="98"/>
+      <c r="B85" s="98"/>
     </row>
     <row r="86" spans="1:2" ht="17.25">
-      <c r="A86" s="49"/>
-      <c r="B86" s="49"/>
+      <c r="A86" s="98"/>
+      <c r="B86" s="98"/>
     </row>
     <row r="87" spans="1:2" ht="17.25">
-      <c r="A87" s="49"/>
-      <c r="B87" s="49"/>
+      <c r="A87" s="98"/>
+      <c r="B87" s="98"/>
     </row>
     <row r="88" spans="1:2" ht="17.25">
-      <c r="A88" s="49"/>
-      <c r="B88" s="49"/>
+      <c r="A88" s="98"/>
+      <c r="B88" s="98"/>
     </row>
     <row r="89" spans="1:2" ht="17.25">
-      <c r="A89" s="49"/>
-      <c r="B89" s="49"/>
+      <c r="A89" s="98"/>
+      <c r="B89" s="98"/>
     </row>
     <row r="90" spans="1:2" ht="17.25">
-      <c r="A90" s="49"/>
-      <c r="B90" s="49"/>
+      <c r="A90" s="98"/>
+      <c r="B90" s="98"/>
     </row>
     <row r="91" spans="1:2" ht="17.25">
-      <c r="A91" s="49"/>
-      <c r="B91" s="49"/>
+      <c r="A91" s="98"/>
+      <c r="B91" s="98"/>
     </row>
     <row r="92" spans="1:2" ht="17.25">
-      <c r="A92" s="49"/>
-      <c r="B92" s="49"/>
+      <c r="A92" s="98"/>
+      <c r="B92" s="98"/>
     </row>
     <row r="93" spans="1:2" ht="17.25">
-      <c r="A93" s="49"/>
-      <c r="B93" s="49"/>
+      <c r="A93" s="98"/>
+      <c r="B93" s="98"/>
     </row>
     <row r="94" spans="1:2" ht="17.25">
-      <c r="A94" s="49"/>
-      <c r="B94" s="49"/>
+      <c r="A94" s="98"/>
+      <c r="B94" s="98"/>
     </row>
     <row r="95" spans="1:2" ht="17.25">
-      <c r="A95" s="49"/>
-      <c r="B95" s="49"/>
+      <c r="A95" s="98"/>
+      <c r="B95" s="98"/>
     </row>
     <row r="96" spans="1:2" ht="17.25">
-      <c r="A96" s="49"/>
-      <c r="B96" s="49"/>
+      <c r="A96" s="98"/>
+      <c r="B96" s="98"/>
     </row>
     <row r="97" spans="1:2" ht="17.25">
-      <c r="A97" s="49"/>
-      <c r="B97" s="49"/>
+      <c r="A97" s="98"/>
+      <c r="B97" s="98"/>
     </row>
     <row r="98" spans="1:2" ht="17.25">
-      <c r="A98" s="49"/>
-      <c r="B98" s="49"/>
+      <c r="A98" s="98"/>
+      <c r="B98" s="98"/>
     </row>
     <row r="99" spans="1:2" ht="17.25">
-      <c r="A99" s="49"/>
-      <c r="B99" s="49"/>
+      <c r="A99" s="98"/>
+      <c r="B99" s="98"/>
     </row>
     <row r="100" spans="1:2" ht="17.25">
-      <c r="A100" s="49"/>
-      <c r="B100" s="49"/>
+      <c r="A100" s="98"/>
+      <c r="B100" s="98"/>
     </row>
     <row r="101" spans="1:2" ht="17.25">
-      <c r="A101" s="49"/>
-      <c r="B101" s="49"/>
+      <c r="A101" s="98"/>
+      <c r="B101" s="98"/>
     </row>
     <row r="102" spans="1:2" ht="17.25">
-      <c r="A102" s="49"/>
-      <c r="B102" s="49"/>
+      <c r="A102" s="98"/>
+      <c r="B102" s="98"/>
     </row>
     <row r="103" spans="1:2" ht="17.25">
-      <c r="A103" s="49"/>
-      <c r="B103" s="49"/>
+      <c r="A103" s="98"/>
+      <c r="B103" s="98"/>
     </row>
     <row r="104" spans="1:2" ht="17.25">
-      <c r="A104" s="49"/>
-      <c r="B104" s="49"/>
+      <c r="A104" s="98"/>
+      <c r="B104" s="98"/>
     </row>
     <row r="105" spans="1:2" ht="17.25">
-      <c r="A105" s="49"/>
-      <c r="B105" s="49"/>
+      <c r="A105" s="98"/>
+      <c r="B105" s="98"/>
     </row>
     <row r="106" spans="1:2" ht="17.25">
-      <c r="A106" s="49"/>
-      <c r="B106" s="49"/>
+      <c r="A106" s="98"/>
+      <c r="B106" s="98"/>
     </row>
     <row r="107" spans="1:2" ht="17.25">
-      <c r="A107" s="49"/>
-      <c r="B107" s="49"/>
+      <c r="A107" s="98"/>
+      <c r="B107" s="98"/>
     </row>
     <row r="108" spans="1:2" ht="17.25">
-      <c r="A108" s="49"/>
-      <c r="B108" s="49"/>
+      <c r="A108" s="98"/>
+      <c r="B108" s="98"/>
     </row>
     <row r="109" spans="1:2" ht="17.25">
-      <c r="A109" s="49"/>
-      <c r="B109" s="49"/>
+      <c r="A109" s="98"/>
+      <c r="B109" s="98"/>
     </row>
     <row r="110" spans="1:2" ht="17.25">
-      <c r="A110" s="49"/>
-      <c r="B110" s="49"/>
+      <c r="A110" s="98"/>
+      <c r="B110" s="98"/>
     </row>
     <row r="111" spans="1:2" ht="17.25">
-      <c r="A111" s="49"/>
-      <c r="B111" s="49"/>
+      <c r="A111" s="98"/>
+      <c r="B111" s="98"/>
     </row>
     <row r="112" spans="1:2" ht="17.25">
-      <c r="A112" s="49"/>
-      <c r="B112" s="49"/>
+      <c r="A112" s="98"/>
+      <c r="B112" s="98"/>
     </row>
     <row r="113" spans="1:2" ht="17.25">
-      <c r="A113" s="49"/>
-      <c r="B113" s="49"/>
+      <c r="A113" s="98"/>
+      <c r="B113" s="98"/>
     </row>
     <row r="114" spans="1:2" ht="17.25">
-      <c r="A114" s="49"/>
-      <c r="B114" s="49"/>
+      <c r="A114" s="98"/>
+      <c r="B114" s="98"/>
     </row>
     <row r="115" spans="1:2" ht="17.25">
-      <c r="A115" s="49"/>
-      <c r="B115" s="49"/>
+      <c r="A115" s="98"/>
+      <c r="B115" s="98"/>
     </row>
     <row r="116" spans="1:2" ht="17.25">
-      <c r="A116" s="49"/>
-      <c r="B116" s="49"/>
+      <c r="A116" s="98"/>
+      <c r="B116" s="98"/>
     </row>
     <row r="117" spans="1:2" ht="17.25">
-      <c r="A117" s="49"/>
-      <c r="B117" s="49"/>
+      <c r="A117" s="98"/>
+      <c r="B117" s="98"/>
     </row>
     <row r="118" spans="1:2" ht="17.25">
-      <c r="A118" s="49"/>
-      <c r="B118" s="49"/>
+      <c r="A118" s="98"/>
+      <c r="B118" s="98"/>
     </row>
     <row r="119" spans="1:2" ht="17.25">
-      <c r="A119" s="49"/>
-      <c r="B119" s="49"/>
+      <c r="A119" s="98"/>
+      <c r="B119" s="98"/>
     </row>
     <row r="120" spans="1:2" ht="17.25">
-      <c r="A120" s="49"/>
-      <c r="B120" s="49"/>
+      <c r="A120" s="98"/>
+      <c r="B120" s="98"/>
     </row>
     <row r="121" spans="1:2" ht="17.25">
-      <c r="A121" s="49"/>
-      <c r="B121" s="49"/>
+      <c r="A121" s="98"/>
+      <c r="B121" s="98"/>
     </row>
     <row r="122" spans="1:2" ht="17.25">
-      <c r="A122" s="49"/>
-      <c r="B122" s="49"/>
+      <c r="A122" s="98"/>
+      <c r="B122" s="98"/>
     </row>
     <row r="123" spans="1:2" ht="17.25">
-      <c r="A123" s="49"/>
-      <c r="B123" s="49"/>
+      <c r="A123" s="98"/>
+      <c r="B123" s="98"/>
     </row>
     <row r="124" spans="1:2" ht="17.25">
-      <c r="A124" s="49"/>
-      <c r="B124" s="49"/>
+      <c r="A124" s="98"/>
+      <c r="B124" s="98"/>
     </row>
     <row r="125" spans="1:2" ht="17.25">
-      <c r="A125" s="49"/>
-      <c r="B125" s="49"/>
+      <c r="A125" s="98"/>
+      <c r="B125" s="98"/>
     </row>
     <row r="126" spans="1:2" ht="17.25">
-      <c r="A126" s="49"/>
-      <c r="B126" s="49"/>
+      <c r="A126" s="98"/>
+      <c r="B126" s="98"/>
     </row>
     <row r="127" spans="1:2" ht="17.25">
-      <c r="A127" s="49"/>
-      <c r="B127" s="49"/>
+      <c r="A127" s="98"/>
+      <c r="B127" s="98"/>
     </row>
     <row r="128" spans="1:2" ht="17.25">
-      <c r="A128" s="49"/>
-      <c r="B128" s="49"/>
+      <c r="A128" s="98"/>
+      <c r="B128" s="98"/>
     </row>
     <row r="129" spans="1:2" ht="17.25">
-      <c r="A129" s="49"/>
-      <c r="B129" s="49"/>
+      <c r="A129" s="98"/>
+      <c r="B129" s="98"/>
     </row>
     <row r="130" spans="1:2" ht="17.25">
-      <c r="A130" s="49"/>
-      <c r="B130" s="49"/>
+      <c r="A130" s="98"/>
+      <c r="B130" s="98"/>
     </row>
     <row r="131" spans="1:2" ht="17.25">
-      <c r="A131" s="49"/>
-      <c r="B131" s="49"/>
+      <c r="A131" s="98"/>
+      <c r="B131" s="98"/>
     </row>
     <row r="132" spans="1:2" ht="17.25">
-      <c r="A132" s="49"/>
-      <c r="B132" s="49"/>
+      <c r="A132" s="98"/>
+      <c r="B132" s="98"/>
     </row>
     <row r="133" spans="1:2" ht="17.25">
-      <c r="A133" s="49"/>
-      <c r="B133" s="49"/>
+      <c r="A133" s="98"/>
+      <c r="B133" s="98"/>
     </row>
     <row r="134" spans="1:2" ht="17.25">
-      <c r="A134" s="49"/>
-      <c r="B134" s="49"/>
+      <c r="A134" s="98"/>
+      <c r="B134" s="98"/>
     </row>
     <row r="135" spans="1:2" ht="17.25">
-      <c r="A135" s="49"/>
-      <c r="B135" s="49"/>
+      <c r="A135" s="98"/>
+      <c r="B135" s="98"/>
     </row>
     <row r="136" spans="1:2" ht="17.25">
-      <c r="A136" s="49"/>
-      <c r="B136" s="49"/>
+      <c r="A136" s="98"/>
+      <c r="B136" s="98"/>
     </row>
     <row r="137" spans="1:2" ht="17.25">
-      <c r="A137" s="49"/>
-      <c r="B137" s="49"/>
+      <c r="A137" s="98"/>
+      <c r="B137" s="98"/>
     </row>
     <row r="138" spans="1:2" ht="17.25">
-      <c r="A138" s="49"/>
-      <c r="B138" s="49"/>
+      <c r="A138" s="98"/>
+      <c r="B138" s="98"/>
     </row>
     <row r="139" spans="1:2" ht="17.25">
-      <c r="A139" s="49"/>
-      <c r="B139" s="49"/>
+      <c r="A139" s="98"/>
+      <c r="B139" s="98"/>
     </row>
     <row r="140" spans="1:2" ht="17.25">
-      <c r="A140" s="49"/>
-      <c r="B140" s="49"/>
+      <c r="A140" s="98"/>
+      <c r="B140" s="98"/>
     </row>
     <row r="141" spans="1:2" ht="17.25">
-      <c r="A141" s="49"/>
-      <c r="B141" s="49"/>
+      <c r="A141" s="98"/>
+      <c r="B141" s="98"/>
     </row>
     <row r="142" spans="1:2" ht="17.25">
-      <c r="A142" s="49"/>
-      <c r="B142" s="49"/>
+      <c r="A142" s="98"/>
+      <c r="B142" s="98"/>
     </row>
     <row r="143" spans="1:2" ht="17.25">
-      <c r="A143" s="49"/>
-      <c r="B143" s="49"/>
+      <c r="A143" s="98"/>
+      <c r="B143" s="98"/>
     </row>
     <row r="144" spans="1:2" ht="17.25">
-      <c r="A144" s="49"/>
-      <c r="B144" s="49"/>
+      <c r="A144" s="98"/>
+      <c r="B144" s="98"/>
     </row>
     <row r="145" spans="1:2" ht="17.25">
-      <c r="A145" s="49"/>
-      <c r="B145" s="49"/>
+      <c r="A145" s="98"/>
+      <c r="B145" s="98"/>
     </row>
     <row r="146" spans="1:2" ht="17.25">
-      <c r="A146" s="49"/>
-      <c r="B146" s="49"/>
+      <c r="A146" s="98"/>
+      <c r="B146" s="98"/>
     </row>
     <row r="147" spans="1:2" ht="17.25">
-      <c r="A147" s="49"/>
-      <c r="B147" s="49"/>
+      <c r="A147" s="98"/>
+      <c r="B147" s="98"/>
     </row>
     <row r="148" spans="1:2" ht="17.25">
-      <c r="A148" s="49"/>
-      <c r="B148" s="49"/>
+      <c r="A148" s="98"/>
+      <c r="B148" s="98"/>
     </row>
     <row r="149" spans="1:2" ht="17.25">
-      <c r="A149" s="49"/>
-      <c r="B149" s="49"/>
+      <c r="A149" s="98"/>
+      <c r="B149" s="98"/>
     </row>
     <row r="150" spans="1:2" ht="17.25">
-      <c r="A150" s="49"/>
-      <c r="B150" s="49"/>
+      <c r="A150" s="98"/>
+      <c r="B150" s="98"/>
     </row>
     <row r="151" spans="1:2" ht="17.25">
-      <c r="A151" s="49"/>
-      <c r="B151" s="49"/>
+      <c r="A151" s="98"/>
+      <c r="B151" s="98"/>
     </row>
     <row r="152" spans="1:2" ht="17.25">
-      <c r="A152" s="49"/>
-      <c r="B152" s="49"/>
+      <c r="A152" s="98"/>
+      <c r="B152" s="98"/>
     </row>
     <row r="153" spans="1:2" ht="17.25">
-      <c r="A153" s="49"/>
-      <c r="B153" s="49"/>
+      <c r="A153" s="98"/>
+      <c r="B153" s="98"/>
     </row>
     <row r="154" spans="1:2" ht="17.25">
-      <c r="A154" s="49"/>
-      <c r="B154" s="49"/>
+      <c r="A154" s="98"/>
+      <c r="B154" s="98"/>
     </row>
     <row r="155" spans="1:2" ht="17.25">
-      <c r="A155" s="49"/>
-      <c r="B155" s="49"/>
+      <c r="A155" s="98"/>
+      <c r="B155" s="98"/>
     </row>
     <row r="156" spans="1:2" ht="17.25">
-      <c r="A156" s="49"/>
-      <c r="B156" s="49"/>
+      <c r="A156" s="98"/>
+      <c r="B156" s="98"/>
     </row>
     <row r="157" spans="1:2" ht="17.25">
-      <c r="A157" s="49"/>
-      <c r="B157" s="49"/>
+      <c r="A157" s="98"/>
+      <c r="B157" s="98"/>
     </row>
     <row r="158" spans="1:2" ht="17.25">
-      <c r="A158" s="49"/>
-      <c r="B158" s="49"/>
+      <c r="A158" s="98"/>
+      <c r="B158" s="98"/>
     </row>
     <row r="159" spans="1:2" ht="17.25">
-      <c r="A159" s="49"/>
-      <c r="B159" s="49"/>
+      <c r="A159" s="98"/>
+      <c r="B159" s="98"/>
     </row>
     <row r="160" spans="1:2" ht="17.25">
-      <c r="A160" s="49"/>
-      <c r="B160" s="49"/>
+      <c r="A160" s="98"/>
+      <c r="B160" s="98"/>
     </row>
     <row r="161" spans="1:2" ht="17.25">
-      <c r="A161" s="49"/>
-      <c r="B161" s="49"/>
+      <c r="A161" s="98"/>
+      <c r="B161" s="98"/>
     </row>
     <row r="162" spans="1:2" ht="17.25">
-      <c r="A162" s="49"/>
-      <c r="B162" s="49"/>
+      <c r="A162" s="98"/>
+      <c r="B162" s="98"/>
     </row>
     <row r="163" spans="1:2" ht="17.25">
-      <c r="A163" s="49"/>
-      <c r="B163" s="49"/>
+      <c r="A163" s="98"/>
+      <c r="B163" s="98"/>
     </row>
     <row r="164" spans="1:2" ht="17.25">
-      <c r="A164" s="49"/>
-      <c r="B164" s="49"/>
+      <c r="A164" s="98"/>
+      <c r="B164" s="98"/>
     </row>
     <row r="165" spans="1:2" ht="17.25">
-      <c r="A165" s="49"/>
-      <c r="B165" s="49"/>
+      <c r="A165" s="98"/>
+      <c r="B165" s="98"/>
     </row>
     <row r="166" spans="1:2" ht="17.25">
-      <c r="A166" s="49"/>
-      <c r="B166" s="49"/>
+      <c r="A166" s="98"/>
+      <c r="B166" s="98"/>
     </row>
     <row r="167" spans="1:2" ht="17.25">
-      <c r="A167" s="49"/>
-      <c r="B167" s="49"/>
+      <c r="A167" s="98"/>
+      <c r="B167" s="98"/>
     </row>
     <row r="168" spans="1:2" ht="17.25">
-      <c r="A168" s="49"/>
-      <c r="B168" s="49"/>
+      <c r="A168" s="98"/>
+      <c r="B168" s="98"/>
     </row>
     <row r="169" spans="1:2" ht="17.25">
-      <c r="A169" s="49"/>
-      <c r="B169" s="49"/>
+      <c r="A169" s="98"/>
+      <c r="B169" s="98"/>
     </row>
     <row r="170" spans="1:2" ht="17.25">
-      <c r="A170" s="49"/>
-      <c r="B170" s="49"/>
+      <c r="A170" s="98"/>
+      <c r="B170" s="98"/>
     </row>
     <row r="171" spans="1:2" ht="17.25">
-      <c r="A171" s="49"/>
-      <c r="B171" s="49"/>
+      <c r="A171" s="98"/>
+      <c r="B171" s="98"/>
     </row>
     <row r="172" spans="1:2" ht="17.25">
-      <c r="A172" s="49"/>
-      <c r="B172" s="49"/>
+      <c r="A172" s="98"/>
+      <c r="B172" s="98"/>
     </row>
     <row r="173" spans="1:2" ht="17.25">
-      <c r="A173" s="49"/>
-      <c r="B173" s="49"/>
+      <c r="A173" s="98"/>
+      <c r="B173" s="98"/>
     </row>
     <row r="174" spans="1:2" ht="17.25">
-      <c r="A174" s="49"/>
-      <c r="B174" s="49"/>
+      <c r="A174" s="98"/>
+      <c r="B174" s="98"/>
     </row>
     <row r="175" spans="1:2" ht="17.25">
-      <c r="A175" s="49"/>
-      <c r="B175" s="49"/>
+      <c r="A175" s="98"/>
+      <c r="B175" s="98"/>
     </row>
     <row r="176" spans="1:2" ht="17.25">
-      <c r="A176" s="49"/>
-      <c r="B176" s="49"/>
+      <c r="A176" s="98"/>
+      <c r="B176" s="98"/>
     </row>
     <row r="177" spans="1:2" ht="17.25">
-      <c r="A177" s="49"/>
-      <c r="B177" s="49"/>
+      <c r="A177" s="98"/>
+      <c r="B177" s="98"/>
     </row>
     <row r="178" spans="1:2" ht="17.25">
-      <c r="A178" s="49"/>
-      <c r="B178" s="49"/>
+      <c r="A178" s="98"/>
+      <c r="B178" s="98"/>
     </row>
     <row r="179" spans="1:2" ht="17.25">
-      <c r="A179" s="49"/>
-      <c r="B179" s="49"/>
+      <c r="A179" s="98"/>
+      <c r="B179" s="98"/>
     </row>
     <row r="180" spans="1:2" ht="17.25">
-      <c r="A180" s="49"/>
-      <c r="B180" s="49"/>
+      <c r="A180" s="98"/>
+      <c r="B180" s="98"/>
     </row>
     <row r="181" spans="1:2" ht="17.25">
-      <c r="A181" s="49"/>
-      <c r="B181" s="49"/>
+      <c r="A181" s="98"/>
+      <c r="B181" s="98"/>
     </row>
     <row r="182" spans="1:2" ht="17.25">
-      <c r="A182" s="49"/>
-      <c r="B182" s="49"/>
+      <c r="A182" s="98"/>
+      <c r="B182" s="98"/>
     </row>
     <row r="183" spans="1:2" ht="17.25">
-      <c r="A183" s="49"/>
-      <c r="B183" s="49"/>
+      <c r="A183" s="98"/>
+      <c r="B183" s="98"/>
     </row>
     <row r="184" spans="1:2" ht="17.25">
-      <c r="A184" s="49"/>
-      <c r="B184" s="49"/>
+      <c r="A184" s="98"/>
+      <c r="B184" s="98"/>
     </row>
     <row r="185" spans="1:2" ht="17.25">
-      <c r="A185" s="49"/>
-      <c r="B185" s="49"/>
+      <c r="A185" s="98"/>
+      <c r="B185" s="98"/>
     </row>
     <row r="186" spans="1:2" ht="17.25">
-      <c r="A186" s="49"/>
-      <c r="B186" s="49"/>
+      <c r="A186" s="98"/>
+      <c r="B186" s="98"/>
     </row>
     <row r="187" spans="1:2" ht="17.25">
-      <c r="A187" s="49"/>
-      <c r="B187" s="49"/>
+      <c r="A187" s="98"/>
+      <c r="B187" s="98"/>
     </row>
     <row r="188" spans="1:2" ht="17.25">
-      <c r="A188" s="49"/>
-      <c r="B188" s="49"/>
+      <c r="A188" s="98"/>
+      <c r="B188" s="98"/>
     </row>
     <row r="189" spans="1:2" ht="17.25">
-      <c r="A189" s="49"/>
-      <c r="B189" s="49"/>
+      <c r="A189" s="98"/>
+      <c r="B189" s="98"/>
     </row>
     <row r="190" spans="1:2" ht="17.25">
-      <c r="A190" s="49"/>
-      <c r="B190" s="49"/>
+      <c r="A190" s="98"/>
+      <c r="B190" s="98"/>
     </row>
     <row r="191" spans="1:2" ht="17.25">
-      <c r="A191" s="49"/>
-      <c r="B191" s="49"/>
+      <c r="A191" s="98"/>
+      <c r="B191" s="98"/>
     </row>
     <row r="192" spans="1:2" ht="17.25">
-      <c r="A192" s="49"/>
-      <c r="B192" s="49"/>
+      <c r="A192" s="98"/>
+      <c r="B192" s="98"/>
     </row>
     <row r="193" spans="1:2" ht="17.25">
-      <c r="A193" s="49"/>
-      <c r="B193" s="49"/>
+      <c r="A193" s="98"/>
+      <c r="B193" s="98"/>
     </row>
     <row r="194" spans="1:2" ht="17.25">
-      <c r="A194" s="49"/>
-      <c r="B194" s="49"/>
+      <c r="A194" s="98"/>
+      <c r="B194" s="98"/>
     </row>
     <row r="195" spans="1:2" ht="17.25">
-      <c r="A195" s="49"/>
-      <c r="B195" s="49"/>
+      <c r="A195" s="98"/>
+      <c r="B195" s="98"/>
     </row>
     <row r="196" spans="1:2" ht="17.25">
-      <c r="A196" s="49"/>
-      <c r="B196" s="49"/>
+      <c r="A196" s="98"/>
+      <c r="B196" s="98"/>
     </row>
     <row r="197" spans="1:2" ht="17.25">
-      <c r="A197" s="49"/>
-      <c r="B197" s="49"/>
+      <c r="A197" s="98"/>
+      <c r="B197" s="98"/>
     </row>
   </sheetData>
   <mergeCells count="147">
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A62:B62"/>
+    <mergeCell ref="A63:B63"/>
+    <mergeCell ref="A58:B58"/>
+    <mergeCell ref="A59:B59"/>
+    <mergeCell ref="A60:B60"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A75:B75"/>
+    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="A71:B71"/>
+    <mergeCell ref="A72:B72"/>
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A82:B82"/>
+    <mergeCell ref="A83:B83"/>
+    <mergeCell ref="A84:B84"/>
+    <mergeCell ref="A79:B79"/>
+    <mergeCell ref="A80:B80"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="A77:B77"/>
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="A91:B91"/>
+    <mergeCell ref="A92:B92"/>
+    <mergeCell ref="A93:B93"/>
+    <mergeCell ref="A88:B88"/>
+    <mergeCell ref="A89:B89"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="A85:B85"/>
+    <mergeCell ref="A86:B86"/>
+    <mergeCell ref="A87:B87"/>
+    <mergeCell ref="A100:B100"/>
+    <mergeCell ref="A101:B101"/>
+    <mergeCell ref="A102:B102"/>
+    <mergeCell ref="A97:B97"/>
+    <mergeCell ref="A98:B98"/>
+    <mergeCell ref="A99:B99"/>
+    <mergeCell ref="A94:B94"/>
+    <mergeCell ref="A95:B95"/>
+    <mergeCell ref="A96:B96"/>
+    <mergeCell ref="A109:B109"/>
+    <mergeCell ref="A110:B110"/>
+    <mergeCell ref="A111:B111"/>
+    <mergeCell ref="A106:B106"/>
+    <mergeCell ref="A107:B107"/>
+    <mergeCell ref="A108:B108"/>
+    <mergeCell ref="A103:B103"/>
+    <mergeCell ref="A104:B104"/>
+    <mergeCell ref="A105:B105"/>
+    <mergeCell ref="A118:B118"/>
+    <mergeCell ref="A119:B119"/>
+    <mergeCell ref="A120:B120"/>
+    <mergeCell ref="A115:B115"/>
+    <mergeCell ref="A116:B116"/>
+    <mergeCell ref="A117:B117"/>
+    <mergeCell ref="A112:B112"/>
+    <mergeCell ref="A113:B113"/>
+    <mergeCell ref="A114:B114"/>
+    <mergeCell ref="A127:B127"/>
+    <mergeCell ref="A128:B128"/>
+    <mergeCell ref="A129:B129"/>
+    <mergeCell ref="A124:B124"/>
+    <mergeCell ref="A125:B125"/>
+    <mergeCell ref="A126:B126"/>
+    <mergeCell ref="A121:B121"/>
+    <mergeCell ref="A122:B122"/>
+    <mergeCell ref="A123:B123"/>
+    <mergeCell ref="A136:B136"/>
+    <mergeCell ref="A137:B137"/>
+    <mergeCell ref="A138:B138"/>
+    <mergeCell ref="A133:B133"/>
+    <mergeCell ref="A134:B134"/>
+    <mergeCell ref="A135:B135"/>
+    <mergeCell ref="A130:B130"/>
+    <mergeCell ref="A131:B131"/>
+    <mergeCell ref="A132:B132"/>
+    <mergeCell ref="A145:B145"/>
+    <mergeCell ref="A146:B146"/>
+    <mergeCell ref="A147:B147"/>
+    <mergeCell ref="A142:B142"/>
+    <mergeCell ref="A143:B143"/>
+    <mergeCell ref="A144:B144"/>
+    <mergeCell ref="A139:B139"/>
+    <mergeCell ref="A140:B140"/>
+    <mergeCell ref="A141:B141"/>
+    <mergeCell ref="A154:B154"/>
+    <mergeCell ref="A155:B155"/>
+    <mergeCell ref="A156:B156"/>
+    <mergeCell ref="A151:B151"/>
+    <mergeCell ref="A152:B152"/>
+    <mergeCell ref="A153:B153"/>
+    <mergeCell ref="A148:B148"/>
+    <mergeCell ref="A149:B149"/>
+    <mergeCell ref="A150:B150"/>
+    <mergeCell ref="A163:B163"/>
+    <mergeCell ref="A164:B164"/>
+    <mergeCell ref="A165:B165"/>
+    <mergeCell ref="A160:B160"/>
+    <mergeCell ref="A161:B161"/>
+    <mergeCell ref="A162:B162"/>
+    <mergeCell ref="A157:B157"/>
+    <mergeCell ref="A158:B158"/>
+    <mergeCell ref="A159:B159"/>
+    <mergeCell ref="A177:B177"/>
+    <mergeCell ref="A172:B172"/>
+    <mergeCell ref="A173:B173"/>
+    <mergeCell ref="A174:B174"/>
+    <mergeCell ref="A169:B169"/>
+    <mergeCell ref="A170:B170"/>
+    <mergeCell ref="A171:B171"/>
+    <mergeCell ref="A166:B166"/>
+    <mergeCell ref="A167:B167"/>
+    <mergeCell ref="A168:B168"/>
     <mergeCell ref="A196:B196"/>
     <mergeCell ref="A197:B197"/>
     <mergeCell ref="B3:G3"/>
@@ -3247,129 +3387,6 @@
     <mergeCell ref="A180:B180"/>
     <mergeCell ref="A175:B175"/>
     <mergeCell ref="A176:B176"/>
-    <mergeCell ref="A177:B177"/>
-    <mergeCell ref="A172:B172"/>
-    <mergeCell ref="A173:B173"/>
-    <mergeCell ref="A174:B174"/>
-    <mergeCell ref="A169:B169"/>
-    <mergeCell ref="A170:B170"/>
-    <mergeCell ref="A171:B171"/>
-    <mergeCell ref="A166:B166"/>
-    <mergeCell ref="A167:B167"/>
-    <mergeCell ref="A168:B168"/>
-    <mergeCell ref="A163:B163"/>
-    <mergeCell ref="A164:B164"/>
-    <mergeCell ref="A165:B165"/>
-    <mergeCell ref="A160:B160"/>
-    <mergeCell ref="A161:B161"/>
-    <mergeCell ref="A162:B162"/>
-    <mergeCell ref="A157:B157"/>
-    <mergeCell ref="A158:B158"/>
-    <mergeCell ref="A159:B159"/>
-    <mergeCell ref="A154:B154"/>
-    <mergeCell ref="A155:B155"/>
-    <mergeCell ref="A156:B156"/>
-    <mergeCell ref="A151:B151"/>
-    <mergeCell ref="A152:B152"/>
-    <mergeCell ref="A153:B153"/>
-    <mergeCell ref="A148:B148"/>
-    <mergeCell ref="A149:B149"/>
-    <mergeCell ref="A150:B150"/>
-    <mergeCell ref="A145:B145"/>
-    <mergeCell ref="A146:B146"/>
-    <mergeCell ref="A147:B147"/>
-    <mergeCell ref="A142:B142"/>
-    <mergeCell ref="A143:B143"/>
-    <mergeCell ref="A144:B144"/>
-    <mergeCell ref="A139:B139"/>
-    <mergeCell ref="A140:B140"/>
-    <mergeCell ref="A141:B141"/>
-    <mergeCell ref="A136:B136"/>
-    <mergeCell ref="A137:B137"/>
-    <mergeCell ref="A138:B138"/>
-    <mergeCell ref="A133:B133"/>
-    <mergeCell ref="A134:B134"/>
-    <mergeCell ref="A135:B135"/>
-    <mergeCell ref="A130:B130"/>
-    <mergeCell ref="A131:B131"/>
-    <mergeCell ref="A132:B132"/>
-    <mergeCell ref="A127:B127"/>
-    <mergeCell ref="A128:B128"/>
-    <mergeCell ref="A129:B129"/>
-    <mergeCell ref="A124:B124"/>
-    <mergeCell ref="A125:B125"/>
-    <mergeCell ref="A126:B126"/>
-    <mergeCell ref="A121:B121"/>
-    <mergeCell ref="A122:B122"/>
-    <mergeCell ref="A123:B123"/>
-    <mergeCell ref="A118:B118"/>
-    <mergeCell ref="A119:B119"/>
-    <mergeCell ref="A120:B120"/>
-    <mergeCell ref="A115:B115"/>
-    <mergeCell ref="A116:B116"/>
-    <mergeCell ref="A117:B117"/>
-    <mergeCell ref="A112:B112"/>
-    <mergeCell ref="A113:B113"/>
-    <mergeCell ref="A114:B114"/>
-    <mergeCell ref="A109:B109"/>
-    <mergeCell ref="A110:B110"/>
-    <mergeCell ref="A111:B111"/>
-    <mergeCell ref="A106:B106"/>
-    <mergeCell ref="A107:B107"/>
-    <mergeCell ref="A108:B108"/>
-    <mergeCell ref="A103:B103"/>
-    <mergeCell ref="A104:B104"/>
-    <mergeCell ref="A105:B105"/>
-    <mergeCell ref="A100:B100"/>
-    <mergeCell ref="A101:B101"/>
-    <mergeCell ref="A102:B102"/>
-    <mergeCell ref="A97:B97"/>
-    <mergeCell ref="A98:B98"/>
-    <mergeCell ref="A99:B99"/>
-    <mergeCell ref="A94:B94"/>
-    <mergeCell ref="A95:B95"/>
-    <mergeCell ref="A96:B96"/>
-    <mergeCell ref="A91:B91"/>
-    <mergeCell ref="A92:B92"/>
-    <mergeCell ref="A93:B93"/>
-    <mergeCell ref="A88:B88"/>
-    <mergeCell ref="A89:B89"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="A85:B85"/>
-    <mergeCell ref="A86:B86"/>
-    <mergeCell ref="A87:B87"/>
-    <mergeCell ref="A82:B82"/>
-    <mergeCell ref="A83:B83"/>
-    <mergeCell ref="A84:B84"/>
-    <mergeCell ref="A79:B79"/>
-    <mergeCell ref="A80:B80"/>
-    <mergeCell ref="A81:B81"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="A77:B77"/>
-    <mergeCell ref="A78:B78"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="A75:B75"/>
-    <mergeCell ref="A70:B70"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="A72:B72"/>
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="B6:G6"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A64:B64"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A62:B62"/>
-    <mergeCell ref="A63:B63"/>
-    <mergeCell ref="A58:B58"/>
-    <mergeCell ref="A59:B59"/>
-    <mergeCell ref="A60:B60"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="H4" r:id="rId1" xr:uid="{45EB914D-0A15-455D-9D63-DC6A78F11C10}"/>
@@ -3387,7 +3404,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.42578125" style="6" customWidth="1"/>
-    <col min="2" max="2" width="61.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="86.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="8" width="28.5703125" style="6" customWidth="1"/>
     <col min="9" max="9" width="4" style="6" customWidth="1"/>
     <col min="10" max="15" width="7.140625" style="6" customWidth="1"/>
@@ -3473,22 +3490,22 @@
       <c r="J6" s="10"/>
     </row>
     <row r="7" spans="1:21" ht="17.100000000000001" customHeight="1" thickBot="1">
-      <c r="C7" s="69" t="s">
+      <c r="C7" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="69" t="s">
+      <c r="D7" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="69" t="s">
+      <c r="E7" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="F7" s="69" t="s">
+      <c r="F7" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="G7" s="69" t="s">
+      <c r="G7" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="H7" s="69" t="s">
+      <c r="H7" s="54" t="s">
         <v>2</v>
       </c>
       <c r="J7" s="6" t="s">
@@ -3497,114 +3514,109 @@
     </row>
     <row r="8" spans="1:21" s="12" customFormat="1" ht="18.75" customHeight="1">
       <c r="A8" s="6"/>
-      <c r="B8" s="88" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="107" t="s">
+      <c r="B8" s="72" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="91" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="107" t="s">
+      <c r="D8" s="91" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="107" t="s">
+      <c r="E8" s="91" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="107" t="s">
+      <c r="F8" s="91" t="s">
         <v>7</v>
       </c>
-      <c r="G8" s="107" t="s">
+      <c r="G8" s="91" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="108" t="s">
+      <c r="H8" s="92" t="s">
         <v>9</v>
       </c>
-      <c r="I8" s="62"/>
-      <c r="J8" s="63">
+      <c r="J8" s="49">
         <v>2027</v>
       </c>
-      <c r="K8" s="63">
+      <c r="K8" s="49">
         <v>2028</v>
       </c>
-      <c r="L8" s="63">
+      <c r="L8" s="49">
         <v>2029</v>
       </c>
-      <c r="M8" s="63">
+      <c r="M8" s="49">
         <v>2030</v>
       </c>
-      <c r="N8" s="63">
+      <c r="N8" s="49">
         <v>2031</v>
       </c>
-      <c r="O8" s="63">
+      <c r="O8" s="49">
         <v>2032</v>
       </c>
-      <c r="P8" s="62"/>
-      <c r="Q8" s="64"/>
-      <c r="R8" s="64"/>
-      <c r="S8" s="64"/>
-      <c r="T8" s="64"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="6"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
       <c r="U8" s="6"/>
     </row>
     <row r="9" spans="1:21" s="12" customFormat="1" ht="18.75" customHeight="1" thickBot="1">
       <c r="A9" s="6"/>
-      <c r="B9" s="100" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="70" t="s">
+      <c r="B9" s="84" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="70" t="s">
+      <c r="D9" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="70" t="s">
+      <c r="E9" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="70" t="s">
+      <c r="F9" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="70" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" s="109" t="s">
+      <c r="G9" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="H9" s="93" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="62"/>
-      <c r="J9" s="63"/>
-      <c r="K9" s="63"/>
-      <c r="L9" s="63"/>
-      <c r="M9" s="63"/>
-      <c r="N9" s="63"/>
-      <c r="O9" s="63"/>
-      <c r="P9" s="62"/>
-      <c r="Q9" s="64"/>
-      <c r="R9" s="64"/>
-      <c r="S9" s="64"/>
-      <c r="T9" s="64"/>
+      <c r="J9" s="49"/>
+      <c r="K9" s="49"/>
+      <c r="L9" s="49"/>
+      <c r="M9" s="49"/>
+      <c r="N9" s="49"/>
+      <c r="O9" s="49"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="6"/>
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
       <c r="U9" s="6"/>
     </row>
     <row r="10" spans="1:21" s="12" customFormat="1" ht="17.25">
       <c r="A10" s="6"/>
-      <c r="B10" s="101" t="s">
+      <c r="B10" s="85" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="93">
+      <c r="C10" s="77">
         <v>123200</v>
       </c>
-      <c r="D10" s="71">
+      <c r="D10" s="56">
         <v>123200</v>
       </c>
-      <c r="E10" s="71">
+      <c r="E10" s="56">
         <v>123200</v>
       </c>
-      <c r="F10" s="71">
+      <c r="F10" s="56">
         <v>123200</v>
       </c>
-      <c r="G10" s="71">
+      <c r="G10" s="56">
         <v>123200</v>
       </c>
-      <c r="H10" s="72">
+      <c r="H10" s="57">
         <v>125600</v>
       </c>
-      <c r="I10" s="62"/>
       <c r="J10" s="36">
         <v>1</v>
       </c>
@@ -3623,7 +3635,6 @@
       <c r="O10" s="36">
         <v>1</v>
       </c>
-      <c r="P10" s="62"/>
       <c r="Q10" s="39" t="s">
         <v>27</v>
       </c>
@@ -3637,10 +3648,10 @@
       <c r="U10" s="6"/>
     </row>
     <row r="11" spans="1:21">
-      <c r="B11" s="102" t="s">
+      <c r="B11" s="86" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="94">
+      <c r="C11" s="78">
         <v>106100</v>
       </c>
       <c r="D11" s="31">
@@ -3655,10 +3666,9 @@
       <c r="G11" s="31">
         <v>106100</v>
       </c>
-      <c r="H11" s="73">
+      <c r="H11" s="58">
         <v>108200</v>
       </c>
-      <c r="I11" s="64"/>
       <c r="J11" s="36">
         <v>1.02</v>
       </c>
@@ -3677,7 +3687,6 @@
       <c r="O11" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P11" s="64"/>
       <c r="Q11" s="43">
         <v>1</v>
       </c>
@@ -3692,10 +3701,10 @@
       </c>
     </row>
     <row r="12" spans="1:21" ht="15.75" thickBot="1">
-      <c r="B12" s="103" t="s">
+      <c r="B12" s="87" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="94">
+      <c r="C12" s="78">
         <v>11000</v>
       </c>
       <c r="D12" s="31">
@@ -3710,10 +3719,9 @@
       <c r="G12" s="31">
         <v>11000</v>
       </c>
-      <c r="H12" s="73">
+      <c r="H12" s="58">
         <v>10000</v>
       </c>
-      <c r="I12" s="64"/>
       <c r="J12" s="36">
         <v>1.02</v>
       </c>
@@ -3732,7 +3740,6 @@
       <c r="O12" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P12" s="64"/>
       <c r="Q12" s="45">
         <v>2</v>
       </c>
@@ -3747,10 +3754,10 @@
       </c>
     </row>
     <row r="13" spans="1:21">
-      <c r="B13" s="103" t="s">
+      <c r="B13" s="87" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="94">
+      <c r="C13" s="78">
         <v>16000</v>
       </c>
       <c r="D13" s="31">
@@ -3765,10 +3772,9 @@
       <c r="G13" s="31">
         <v>16000</v>
       </c>
-      <c r="H13" s="73">
+      <c r="H13" s="58">
         <v>16000</v>
       </c>
-      <c r="I13" s="64"/>
       <c r="J13" s="36">
         <v>1.02</v>
       </c>
@@ -3787,17 +3793,12 @@
       <c r="O13" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P13" s="64"/>
-      <c r="Q13" s="64"/>
-      <c r="R13" s="64"/>
-      <c r="S13" s="64"/>
-      <c r="T13" s="64"/>
     </row>
     <row r="14" spans="1:21">
-      <c r="B14" s="103" t="s">
+      <c r="B14" s="87" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="95">
+      <c r="C14" s="79">
         <v>25000</v>
       </c>
       <c r="D14" s="32">
@@ -3812,10 +3813,9 @@
       <c r="G14" s="32">
         <v>30000</v>
       </c>
-      <c r="H14" s="74">
+      <c r="H14" s="59">
         <v>0</v>
       </c>
-      <c r="I14" s="64"/>
       <c r="J14" s="36">
         <v>1.02</v>
       </c>
@@ -3834,17 +3834,12 @@
       <c r="O14" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P14" s="64"/>
-      <c r="Q14" s="64"/>
-      <c r="R14" s="64"/>
-      <c r="S14" s="64"/>
-      <c r="T14" s="64"/>
     </row>
     <row r="15" spans="1:21">
-      <c r="B15" s="103" t="s">
+      <c r="B15" s="87" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="96">
+      <c r="C15" s="80">
         <v>2000</v>
       </c>
       <c r="D15" s="32">
@@ -3859,10 +3854,9 @@
       <c r="G15" s="33">
         <v>4500</v>
       </c>
-      <c r="H15" s="75">
+      <c r="H15" s="60">
         <v>0</v>
       </c>
-      <c r="I15" s="64"/>
       <c r="J15" s="36">
         <v>1.02</v>
       </c>
@@ -3881,17 +3875,12 @@
       <c r="O15" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P15" s="64"/>
-      <c r="Q15" s="64"/>
-      <c r="R15" s="64"/>
-      <c r="S15" s="64"/>
-      <c r="T15" s="64"/>
     </row>
     <row r="16" spans="1:21">
-      <c r="B16" s="103" t="s">
+      <c r="B16" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="95">
+      <c r="C16" s="79">
         <v>18000</v>
       </c>
       <c r="D16" s="32">
@@ -3906,10 +3895,9 @@
       <c r="G16" s="32">
         <v>18000</v>
       </c>
-      <c r="H16" s="74">
+      <c r="H16" s="59">
         <v>13000</v>
       </c>
-      <c r="I16" s="64"/>
       <c r="J16" s="36">
         <v>1.02</v>
       </c>
@@ -3928,17 +3916,12 @@
       <c r="O16" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P16" s="64"/>
-      <c r="Q16" s="64"/>
-      <c r="R16" s="64"/>
-      <c r="S16" s="64"/>
-      <c r="T16" s="64"/>
-    </row>
-    <row r="17" spans="2:20">
-      <c r="B17" s="103" t="s">
+    </row>
+    <row r="17" spans="2:15">
+      <c r="B17" s="87" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="94">
+      <c r="C17" s="78">
         <v>2000</v>
       </c>
       <c r="D17" s="31">
@@ -3953,10 +3936,9 @@
       <c r="G17" s="31">
         <v>2000</v>
       </c>
-      <c r="H17" s="73">
+      <c r="H17" s="58">
         <v>2000</v>
       </c>
-      <c r="I17" s="64"/>
       <c r="J17" s="36">
         <v>1.02</v>
       </c>
@@ -3975,17 +3957,12 @@
       <c r="O17" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P17" s="64"/>
-      <c r="Q17" s="64"/>
-      <c r="R17" s="64"/>
-      <c r="S17" s="64"/>
-      <c r="T17" s="64"/>
-    </row>
-    <row r="18" spans="2:20">
-      <c r="B18" s="103" t="s">
+    </row>
+    <row r="18" spans="2:15">
+      <c r="B18" s="87" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="96">
+      <c r="C18" s="80">
         <v>450</v>
       </c>
       <c r="D18" s="33">
@@ -4000,10 +3977,9 @@
       <c r="G18" s="33">
         <v>450</v>
       </c>
-      <c r="H18" s="75">
+      <c r="H18" s="60">
         <v>400</v>
       </c>
-      <c r="I18" s="64"/>
       <c r="J18" s="36">
         <v>1.02</v>
       </c>
@@ -4022,17 +3998,12 @@
       <c r="O18" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P18" s="64"/>
-      <c r="Q18" s="64"/>
-      <c r="R18" s="64"/>
-      <c r="S18" s="64"/>
-      <c r="T18" s="64"/>
-    </row>
-    <row r="19" spans="2:20">
-      <c r="B19" s="103" t="s">
+    </row>
+    <row r="19" spans="2:15">
+      <c r="B19" s="87" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="96">
+      <c r="C19" s="80">
         <v>280</v>
       </c>
       <c r="D19" s="33">
@@ -4047,10 +4018,9 @@
       <c r="G19" s="33">
         <v>280</v>
       </c>
-      <c r="H19" s="75">
+      <c r="H19" s="60">
         <v>50</v>
       </c>
-      <c r="I19" s="64"/>
       <c r="J19" s="36">
         <v>1.02</v>
       </c>
@@ -4069,17 +4039,12 @@
       <c r="O19" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P19" s="64"/>
-      <c r="Q19" s="64"/>
-      <c r="R19" s="64"/>
-      <c r="S19" s="64"/>
-      <c r="T19" s="64"/>
-    </row>
-    <row r="20" spans="2:20">
-      <c r="B20" s="104" t="s">
+    </row>
+    <row r="20" spans="2:15">
+      <c r="B20" s="88" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="97">
+      <c r="C20" s="81">
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="D20" s="34">
@@ -4094,10 +4059,9 @@
       <c r="G20" s="34">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="H20" s="76">
+      <c r="H20" s="61">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="I20" s="64"/>
       <c r="J20" s="36">
         <v>1.02</v>
       </c>
@@ -4116,17 +4080,12 @@
       <c r="O20" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P20" s="64"/>
-      <c r="Q20" s="64"/>
-      <c r="R20" s="64"/>
-      <c r="S20" s="64"/>
-      <c r="T20" s="64"/>
-    </row>
-    <row r="21" spans="2:20">
-      <c r="B21" s="103" t="s">
+    </row>
+    <row r="21" spans="2:15">
+      <c r="B21" s="87" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="95">
+      <c r="C21" s="79">
         <v>300</v>
       </c>
       <c r="D21" s="32">
@@ -4141,10 +4100,9 @@
       <c r="G21" s="33">
         <v>3100</v>
       </c>
-      <c r="H21" s="75">
+      <c r="H21" s="60">
         <v>300</v>
       </c>
-      <c r="I21" s="64"/>
       <c r="J21" s="36">
         <v>1.02</v>
       </c>
@@ -4163,41 +4121,29 @@
       <c r="O21" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P21" s="64"/>
-      <c r="Q21" s="64"/>
-      <c r="R21" s="64"/>
-      <c r="S21" s="64"/>
-      <c r="T21" s="64"/>
-    </row>
-    <row r="22" spans="2:20">
-      <c r="B22" s="103" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="94">
-        <f>794.13*80^(-0.61)*1000</f>
-        <v>54828.543692751693</v>
-      </c>
-      <c r="D22" s="31">
-        <f>794.13*80^(-0.61)*1000</f>
-        <v>54828.543692751693</v>
-      </c>
-      <c r="E22" s="31">
-        <f>794.13*80^(-0.61)*1000</f>
-        <v>54828.543692751693</v>
-      </c>
-      <c r="F22" s="31">
-        <f>794.13*80^(-0.61)*1000</f>
-        <v>54828.543692751693</v>
-      </c>
-      <c r="G22" s="31">
-        <f>794.13*80^(-0.61)*1000</f>
-        <v>54828.543692751693</v>
-      </c>
-      <c r="H22" s="73">
-        <f>794.13*80^(-0.61)*1000</f>
-        <v>54828.543692751693</v>
-      </c>
-      <c r="I22" s="64"/>
+    </row>
+    <row r="22" spans="2:15">
+      <c r="B22" s="87" t="s">
+        <v>56</v>
+      </c>
+      <c r="C22" s="111" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" s="112" t="s">
+        <v>54</v>
+      </c>
+      <c r="E22" s="112" t="s">
+        <v>54</v>
+      </c>
+      <c r="F22" s="112" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" s="112" t="s">
+        <v>54</v>
+      </c>
+      <c r="H22" s="113" t="s">
+        <v>54</v>
+      </c>
       <c r="J22" s="36">
         <v>1.02</v>
       </c>
@@ -4216,41 +4162,29 @@
       <c r="O22" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P22" s="64"/>
-      <c r="Q22" s="64"/>
-      <c r="R22" s="64"/>
-      <c r="S22" s="64"/>
-      <c r="T22" s="64"/>
-    </row>
-    <row r="23" spans="2:20" ht="17.100000000000001" customHeight="1">
-      <c r="B23" s="103" t="s">
-        <v>42</v>
-      </c>
-      <c r="C23" s="94">
-        <f>1408*80^(-0.891)*1000</f>
-        <v>28375.888986274687</v>
-      </c>
-      <c r="D23" s="31">
-        <f>1408*80^(-0.891)*1000</f>
-        <v>28375.888986274687</v>
-      </c>
-      <c r="E23" s="31">
-        <f>1408*80^(-0.891)*1000</f>
-        <v>28375.888986274687</v>
-      </c>
-      <c r="F23" s="31">
-        <f>1408*80^(-0.891)*1000</f>
-        <v>28375.888986274687</v>
-      </c>
-      <c r="G23" s="31">
-        <f>1408*80^(-0.891)*1000</f>
-        <v>28375.888986274687</v>
-      </c>
-      <c r="H23" s="73">
-        <f>1408*80^(-0.891)*1000</f>
-        <v>28375.888986274687</v>
-      </c>
-      <c r="I23" s="64"/>
+    </row>
+    <row r="23" spans="2:15" ht="17.100000000000001" customHeight="1">
+      <c r="B23" s="87" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="111" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="112" t="s">
+        <v>55</v>
+      </c>
+      <c r="E23" s="112" t="s">
+        <v>55</v>
+      </c>
+      <c r="F23" s="112" t="s">
+        <v>55</v>
+      </c>
+      <c r="G23" s="112" t="s">
+        <v>55</v>
+      </c>
+      <c r="H23" s="113" t="s">
+        <v>55</v>
+      </c>
       <c r="J23" s="36">
         <v>1.02</v>
       </c>
@@ -4269,17 +4203,12 @@
       <c r="O23" s="36">
         <v>1.1259999999999999</v>
       </c>
-      <c r="P23" s="64"/>
-      <c r="Q23" s="64"/>
-      <c r="R23" s="64"/>
-      <c r="S23" s="64"/>
-      <c r="T23" s="64"/>
-    </row>
-    <row r="24" spans="2:20" ht="17.100000000000001" customHeight="1">
-      <c r="B24" s="105" t="s">
+    </row>
+    <row r="24" spans="2:15" ht="17.100000000000001" customHeight="1">
+      <c r="B24" s="89" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="98">
+      <c r="C24" s="82">
         <v>0.05</v>
       </c>
       <c r="D24" s="35">
@@ -4294,89 +4223,65 @@
       <c r="G24" s="35">
         <v>0.05</v>
       </c>
-      <c r="H24" s="77">
+      <c r="H24" s="62">
         <v>0.05</v>
       </c>
-      <c r="I24" s="64"/>
-      <c r="J24" s="64"/>
-      <c r="K24" s="64"/>
-      <c r="L24" s="64"/>
-      <c r="M24" s="64"/>
-      <c r="N24" s="64"/>
-      <c r="O24" s="64"/>
-      <c r="P24" s="64"/>
-      <c r="Q24" s="64"/>
-      <c r="R24" s="64"/>
-      <c r="S24" s="64"/>
-      <c r="T24" s="64"/>
-    </row>
-    <row r="25" spans="2:20" ht="17.100000000000001" customHeight="1" thickBot="1">
-      <c r="B25" s="106" t="s">
+    </row>
+    <row r="25" spans="2:15" ht="17.100000000000001" customHeight="1" thickBot="1">
+      <c r="B25" s="90" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="99">
+      <c r="C25" s="83">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="D25" s="78">
+      <c r="D25" s="63">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="E25" s="78">
+      <c r="E25" s="63">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="F25" s="78">
+      <c r="F25" s="63">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="G25" s="78">
+      <c r="G25" s="63">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="H25" s="79">
+      <c r="H25" s="64">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="I25" s="64"/>
-      <c r="J25" s="64"/>
-      <c r="K25" s="64"/>
-      <c r="L25" s="64"/>
-      <c r="M25" s="64"/>
-      <c r="N25" s="64"/>
-      <c r="O25" s="64"/>
-      <c r="P25" s="64"/>
-      <c r="Q25" s="64"/>
-      <c r="R25" s="64"/>
-      <c r="S25" s="64"/>
-      <c r="T25" s="64"/>
-    </row>
-    <row r="26" spans="2:20" ht="17.100000000000001" customHeight="1"/>
-    <row r="27" spans="2:20" ht="17.100000000000001" customHeight="1" thickBot="1"/>
-    <row r="28" spans="2:20" ht="17.45" customHeight="1">
-      <c r="B28" s="88" t="s">
+    </row>
+    <row r="26" spans="2:15" ht="17.100000000000001" customHeight="1"/>
+    <row r="27" spans="2:15" ht="17.100000000000001" customHeight="1" thickBot="1"/>
+    <row r="28" spans="2:15" ht="17.45" customHeight="1">
+      <c r="B28" s="72" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="2:15" ht="17.45" customHeight="1" thickBot="1">
+      <c r="B29" s="73" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="2:20" ht="17.45" customHeight="1" thickBot="1">
-      <c r="B29" s="89" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="30" spans="2:20" ht="17.100000000000001" customHeight="1">
-      <c r="B30" s="90" t="s">
+    <row r="30" spans="2:15" ht="17.100000000000001" customHeight="1">
+      <c r="B30" s="74" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="84">
+      <c r="C30" s="68">
         <v>2</v>
       </c>
-      <c r="D30" s="65">
+      <c r="D30" s="50">
         <v>2</v>
       </c>
-      <c r="E30" s="65">
+      <c r="E30" s="50">
         <v>2</v>
       </c>
-      <c r="F30" s="65">
+      <c r="F30" s="50">
         <v>2</v>
       </c>
-      <c r="G30" s="65">
+      <c r="G30" s="50">
         <v>2</v>
       </c>
-      <c r="H30" s="66">
+      <c r="H30" s="51">
         <v>2</v>
       </c>
       <c r="J30" s="13">
@@ -4398,11 +4303,11 @@
         <v>1.1259999999999999</v>
       </c>
     </row>
-    <row r="31" spans="2:20" ht="17.100000000000001" customHeight="1">
-      <c r="B31" s="91" t="s">
-        <v>45</v>
-      </c>
-      <c r="C31" s="85">
+    <row r="31" spans="2:15" ht="17.100000000000001" customHeight="1">
+      <c r="B31" s="75" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="69">
         <v>70</v>
       </c>
       <c r="D31" s="29">
@@ -4417,7 +4322,7 @@
       <c r="G31" s="29">
         <v>70</v>
       </c>
-      <c r="H31" s="67">
+      <c r="H31" s="52">
         <v>70</v>
       </c>
       <c r="J31" s="13">
@@ -4439,11 +4344,11 @@
         <v>1.1259999999999999</v>
       </c>
     </row>
-    <row r="32" spans="2:20" ht="17.100000000000001" customHeight="1">
-      <c r="B32" s="91" t="s">
+    <row r="32" spans="2:15" ht="17.100000000000001" customHeight="1">
+      <c r="B32" s="75" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="86" t="s">
+      <c r="C32" s="70" t="s">
         <v>40</v>
       </c>
       <c r="D32" s="30" t="s">
@@ -4458,7 +4363,7 @@
       <c r="G32" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="H32" s="68" t="s">
+      <c r="H32" s="53" t="s">
         <v>40</v>
       </c>
       <c r="J32" s="13">
@@ -4481,143 +4386,143 @@
       </c>
     </row>
     <row r="33" spans="1:21" ht="17.100000000000001" customHeight="1" thickBot="1">
-      <c r="B33" s="92" t="s">
-        <v>43</v>
-      </c>
-      <c r="C33" s="87" t="s">
-        <v>46</v>
-      </c>
-      <c r="D33" s="82" t="s">
-        <v>46</v>
-      </c>
-      <c r="E33" s="82" t="s">
-        <v>46</v>
-      </c>
-      <c r="F33" s="82" t="s">
-        <v>46</v>
-      </c>
-      <c r="G33" s="82" t="s">
-        <v>46</v>
-      </c>
-      <c r="H33" s="83" t="s">
-        <v>46</v>
+      <c r="B33" s="76" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="71" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" s="66" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="66" t="s">
+        <v>44</v>
+      </c>
+      <c r="F33" s="66" t="s">
+        <v>44</v>
+      </c>
+      <c r="G33" s="66" t="s">
+        <v>44</v>
+      </c>
+      <c r="H33" s="67" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="34" spans="1:21" ht="17.100000000000001" customHeight="1">
-      <c r="A34" s="81"/>
-      <c r="B34" s="81"/>
-      <c r="C34" s="81"/>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="81"/>
-      <c r="G34" s="81"/>
-      <c r="H34" s="81"/>
-      <c r="I34" s="81"/>
-      <c r="J34" s="81"/>
-      <c r="K34" s="81"/>
-      <c r="L34" s="81"/>
-      <c r="M34" s="81"/>
-      <c r="N34" s="81"/>
-      <c r="O34" s="81"/>
-      <c r="P34" s="81"/>
-      <c r="Q34" s="81"/>
-      <c r="R34" s="81"/>
-      <c r="S34" s="81"/>
-      <c r="T34" s="81"/>
-      <c r="U34" s="81"/>
+      <c r="A34" s="65"/>
+      <c r="B34" s="65"/>
+      <c r="C34" s="65"/>
+      <c r="D34" s="65"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="65"/>
+      <c r="G34" s="65"/>
+      <c r="H34" s="65"/>
+      <c r="I34" s="65"/>
+      <c r="J34" s="65"/>
+      <c r="K34" s="65"/>
+      <c r="L34" s="65"/>
+      <c r="M34" s="65"/>
+      <c r="N34" s="65"/>
+      <c r="O34" s="65"/>
+      <c r="P34" s="65"/>
+      <c r="Q34" s="65"/>
+      <c r="R34" s="65"/>
+      <c r="S34" s="65"/>
+      <c r="T34" s="65"/>
+      <c r="U34" s="65"/>
     </row>
     <row r="35" spans="1:21" ht="17.100000000000001" customHeight="1">
-      <c r="A35" s="81"/>
-      <c r="B35" s="81"/>
-      <c r="C35" s="81"/>
-      <c r="D35" s="81"/>
-      <c r="E35" s="81"/>
-      <c r="F35" s="81"/>
-      <c r="G35" s="81"/>
-      <c r="H35" s="81"/>
-      <c r="I35" s="81"/>
-      <c r="J35" s="81"/>
-      <c r="K35" s="81"/>
-      <c r="L35" s="81"/>
-      <c r="M35" s="81"/>
-      <c r="N35" s="81"/>
-      <c r="O35" s="81"/>
-      <c r="P35" s="81"/>
-      <c r="Q35" s="81"/>
-      <c r="R35" s="81"/>
-      <c r="S35" s="81"/>
-      <c r="T35" s="81"/>
-      <c r="U35" s="81"/>
+      <c r="A35" s="65"/>
+      <c r="B35" s="65"/>
+      <c r="C35" s="65"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="65"/>
+      <c r="G35" s="65"/>
+      <c r="H35" s="65"/>
+      <c r="I35" s="65"/>
+      <c r="J35" s="65"/>
+      <c r="K35" s="65"/>
+      <c r="L35" s="65"/>
+      <c r="M35" s="65"/>
+      <c r="N35" s="65"/>
+      <c r="O35" s="65"/>
+      <c r="P35" s="65"/>
+      <c r="Q35" s="65"/>
+      <c r="R35" s="65"/>
+      <c r="S35" s="65"/>
+      <c r="T35" s="65"/>
+      <c r="U35" s="65"/>
     </row>
     <row r="36" spans="1:21" ht="17.100000000000001" customHeight="1" thickBot="1">
-      <c r="B36" s="80" t="s">
-        <v>54</v>
-      </c>
-      <c r="C36" s="81"/>
-      <c r="D36" s="81"/>
-      <c r="E36" s="81"/>
-      <c r="F36" s="81"/>
-      <c r="G36" s="81"/>
-      <c r="H36" s="81"/>
+      <c r="B36" s="55" t="s">
+        <v>52</v>
+      </c>
+      <c r="C36" s="65"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="65"/>
+      <c r="G36" s="65"/>
+      <c r="H36" s="65"/>
     </row>
     <row r="37" spans="1:21" ht="17.100000000000001" customHeight="1" thickBot="1">
-      <c r="B37" s="88" t="s">
-        <v>55</v>
-      </c>
-      <c r="C37" s="81"/>
-      <c r="D37" s="81"/>
-      <c r="E37" s="81"/>
-      <c r="F37" s="81"/>
-      <c r="G37" s="81"/>
-      <c r="H37" s="81"/>
+      <c r="B37" s="72" t="s">
+        <v>53</v>
+      </c>
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
     </row>
     <row r="38" spans="1:21" ht="14.1" customHeight="1" thickBot="1">
-      <c r="B38" s="113" t="s">
+      <c r="B38" s="97" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="94">
+        <v>8</v>
+      </c>
+      <c r="D38" s="95">
+        <v>8</v>
+      </c>
+      <c r="E38" s="95">
+        <v>8</v>
+      </c>
+      <c r="F38" s="95">
+        <v>8</v>
+      </c>
+      <c r="G38" s="95">
+        <v>8</v>
+      </c>
+      <c r="H38" s="96">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:21" ht="15" customHeight="1">
+      <c r="A39" s="65"/>
+      <c r="B39" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="C38" s="110">
-        <v>8</v>
-      </c>
-      <c r="D38" s="111">
-        <v>8</v>
-      </c>
-      <c r="E38" s="111">
-        <v>8</v>
-      </c>
-      <c r="F38" s="111">
-        <v>8</v>
-      </c>
-      <c r="G38" s="111">
-        <v>8</v>
-      </c>
-      <c r="H38" s="112">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="1:21" ht="15" customHeight="1">
-      <c r="A39" s="81"/>
-      <c r="B39" s="81" t="s">
-        <v>49</v>
-      </c>
-      <c r="C39" s="81"/>
-      <c r="D39" s="81"/>
-      <c r="E39" s="81"/>
-      <c r="F39" s="81"/>
-      <c r="G39" s="81"/>
-      <c r="H39" s="81"/>
-      <c r="I39" s="81"/>
-      <c r="J39" s="81"/>
-      <c r="K39" s="81"/>
-      <c r="L39" s="81"/>
-      <c r="M39" s="81"/>
-      <c r="N39" s="81"/>
-      <c r="O39" s="81"/>
-      <c r="P39" s="81"/>
-      <c r="Q39" s="81"/>
-      <c r="R39" s="81"/>
-      <c r="S39" s="81"/>
-      <c r="T39" s="81"/>
-      <c r="U39" s="81"/>
+      <c r="C39" s="65"/>
+      <c r="D39" s="65"/>
+      <c r="E39" s="65"/>
+      <c r="F39" s="65"/>
+      <c r="G39" s="65"/>
+      <c r="H39" s="65"/>
+      <c r="I39" s="65"/>
+      <c r="J39" s="65"/>
+      <c r="K39" s="65"/>
+      <c r="L39" s="65"/>
+      <c r="M39" s="65"/>
+      <c r="N39" s="65"/>
+      <c r="O39" s="65"/>
+      <c r="P39" s="65"/>
+      <c r="Q39" s="65"/>
+      <c r="R39" s="65"/>
+      <c r="S39" s="65"/>
+      <c r="T39" s="65"/>
+      <c r="U39" s="65"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4628,20 +4533,53 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="005e6648-557a-461d-8c6b-56cb21250bc8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_Flow_SignoffStatus xmlns="005e6648-557a-461d-8c6b-56cb21250bc8" xsi:nil="true"/>
-    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Not Started</_Status>
-    <_dlc_DocId xmlns="c8bd6623-0a6a-41b2-880d-a1b0487fc1fe">QE-ICP01-1796277528-427670</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="c8bd6623-0a6a-41b2-880d-a1b0487fc1fe">
-      <Url>https://qenergysolutionsse.sharepoint.com/sites/Mind_Services125/_layouts/15/DocIdRedir.aspx?ID=QE-ICP01-1796277528-427670</Url>
-      <Description>QE-ICP01-1796277528-427670</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4894,53 +4832,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="005e6648-557a-461d-8c6b-56cb21250bc8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_Flow_SignoffStatus xmlns="005e6648-557a-461d-8c6b-56cb21250bc8" xsi:nil="true"/>
+    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Not Started</_Status>
+    <_dlc_DocId xmlns="c8bd6623-0a6a-41b2-880d-a1b0487fc1fe">QE-ICP01-1796277528-427670</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="c8bd6623-0a6a-41b2-880d-a1b0487fc1fe">
+      <Url>https://qenergysolutionsse.sharepoint.com/sites/Mind_Services125/_layouts/15/DocIdRedir.aspx?ID=QE-ICP01-1796277528-427670</Url>
+      <Description>QE-ICP01-1796277528-427670</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4953,19 +4858,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{841AC8F3-80E2-4B1C-97B4-491869C7714B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E595D335-0B08-44E4-A5B5-559EF6C44620}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="c8bd6623-0a6a-41b2-880d-a1b0487fc1fe"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="005e6648-557a-461d-8c6b-56cb21250bc8"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4991,9 +4886,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E595D335-0B08-44E4-A5B5-559EF6C44620}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{841AC8F3-80E2-4B1C-97B4-491869C7714B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="c8bd6623-0a6a-41b2-880d-a1b0487fc1fe"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="005e6648-557a-461d-8c6b-56cb21250bc8"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>